<commit_message>
add import template assets
</commit_message>
<xml_diff>
--- a/ImportTemplate/plant_1.xlsx
+++ b/ImportTemplate/plant_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\biog\biog\ImportTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9984B2ED-35FD-4C67-90B6-15486BA077E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{184B49F7-BD93-4874-B47E-86B0AA0E9C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5989159A-E7FB-42B4-9C9A-65CB7C17A329}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
   <si>
     <t>Template Import เนื้อหา ประเภทพืช</t>
   </si>
@@ -129,9 +129,6 @@
     <t>หากระบุข้อมูลที่อยู่ไม่ครบหรือไม่ถูกต้องจากถูก auto จากพิกัดทันที</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>&lt;ชื่อภาพจาก FileCenter&gt;;</t>
   </si>
   <si>
@@ -148,9 +145,6 @@
   </si>
   <si>
     <t>PENDING, APPROVE, REJECT</t>
-  </si>
-  <si>
-    <t>CCA, CCA</t>
   </si>
   <si>
     <t>แสดง</t>
@@ -184,21 +178,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -206,17 +194,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,207 +540,216 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A1F2B36-8FCD-4776-ADD1-AC8F2EA1C9B7}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:X42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="74.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" customWidth="1"/>
     <col min="3" max="3" width="19.140625" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="29.5703125" customWidth="1"/>
+    <col min="7" max="7" width="32.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" customWidth="1"/>
+    <col min="13" max="13" width="17.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" customWidth="1"/>
+    <col min="16" max="16" width="12.28515625" customWidth="1"/>
+    <col min="18" max="18" width="76" customWidth="1"/>
+    <col min="19" max="19" width="16.7109375" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" customWidth="1"/>
+    <col min="23" max="23" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:24">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="16.5">
-      <c r="A2" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+    </row>
+    <row r="2" spans="1:24" ht="16.5">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24">
+      <c r="A3" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.5">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.5">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.5">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="D3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.5">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="E3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="16.5">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="F3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="16.5">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3"/>
-      <c r="C8" t="s">
+      <c r="G3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="16.5">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3"/>
-    </row>
-    <row r="10" spans="1:3" ht="16.5">
-      <c r="A10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3"/>
-    </row>
-    <row r="11" spans="1:3" ht="16.5">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" spans="1:3" ht="16.5">
-      <c r="A12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="3"/>
-    </row>
-    <row r="13" spans="1:3" ht="16.5">
-      <c r="A13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="L3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N3" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" t="s">
+        <v>35</v>
+      </c>
+      <c r="P3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>35</v>
+      </c>
+      <c r="R3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="16.5">
-      <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="16.5">
-      <c r="A15" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="16.5">
-      <c r="A16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="16.5">
-      <c r="A17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="16.5">
-      <c r="A18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="16.5">
-      <c r="A19" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="S3" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" ht="16.5">
-      <c r="A20" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="T3" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" ht="16.5">
-      <c r="A21" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="U3" t="s">
+        <v>36</v>
+      </c>
+      <c r="W3" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" ht="16.5">
-      <c r="A22" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="16.5">
-      <c r="A23" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="X3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="16.5">
-      <c r="A24" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="16.5">
-      <c r="A25" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>39</v>
-      </c>
+    <row r="35" spans="2:2">
+      <c r="B35" s="4"/>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36" s="4"/>
+    </row>
+    <row r="37" spans="2:2">
+      <c r="B37" s="5"/>
+    </row>
+    <row r="38" spans="2:2">
+      <c r="B38" s="5"/>
+    </row>
+    <row r="39" spans="2:2">
+      <c r="B39" s="5"/>
+    </row>
+    <row r="40" spans="2:2">
+      <c r="B40" s="5"/>
+    </row>
+    <row r="41" spans="2:2">
+      <c r="B41" s="5"/>
+    </row>
+    <row r="42" spans="2:2">
+      <c r="B42" s="4"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:X1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>